<commit_message>
fix component and integration tests
</commit_message>
<xml_diff>
--- a/tests/component/fixtures/sportsmen-import.xlsx
+++ b/tests/component/fixtures/sportsmen-import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roman\Projects\trampolin\trampolin\tests\component\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6957A4E5-8270-4201-ABA5-A44833069287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4241CB23-0DAF-4B33-B5B1-57717DE14024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32415" yWindow="2190" windowWidth="21600" windowHeight="12645" xr2:uid="{9BA29B9D-2A43-4B2D-9B54-E9D70108D4C3}"/>
+    <workbookView xWindow="2970" yWindow="1280" windowWidth="14400" windowHeight="7270" xr2:uid="{9BA29B9D-2A43-4B2D-9B54-E9D70108D4C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Name</t>
   </si>
@@ -47,22 +47,37 @@
     <t>Club</t>
   </si>
   <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Created At</t>
-  </si>
-  <si>
     <t>Charlie</t>
   </si>
   <si>
     <t>Test Club 3</t>
   </si>
   <si>
-    <t>Senior Men</t>
-  </si>
-  <si>
     <t>Test Club 4</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Birthyear</t>
+  </si>
+  <si>
+    <t>Routine</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>W11</t>
+  </si>
+  <si>
+    <t>DMT</t>
   </si>
 </sst>
 </file>
@@ -435,10 +450,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB12B3D-0714-4618-B8B0-B14CE8AACF36}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -446,35 +461,47 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1">
         <v>46055</v>
       </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1">
         <v>46056</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>